<commit_message>
Refine Excel dashboard KPI display
</commit_message>
<xml_diff>
--- a/retail-sales-customer-performance/Retail_Sales_Customer_Performance.xlsx
+++ b/retail-sales-customer-performance/Retail_Sales_Customer_Performance.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R6b1a9dc1cc3e4100"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Trend" sheetId="2" r:id="R7441f1df64374451"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer Segments" sheetId="3" r:id="R1d2bb2e045334093"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Markets &amp; Products" sheetId="4" r:id="Rb4fe6081aed94049"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" r:id="R8d873e00e78b4150"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rcc5c83252d5e442e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Trend" sheetId="2" r:id="R3bc10d92b3854b25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer Segments" sheetId="3" r:id="R0836c69d635847ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Markets &amp; Products" sheetId="4" r:id="Rf911fbf935cb4654"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" r:id="R7247c2bc8b6c4417"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -240,34 +240,6 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Month Start</c:v>
-          </c:tx>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Monthly Trend'!$A$4:$A$16</c:f>
-              <c:strCache>
-                <c:ptCount val="0"/>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'Monthly Trend'!$B$4:$B$16</c:f>
-              <c:numCache>
-                <c:formatCode>mmm yyyy</c:formatCode>
-                <c:ptCount val="0"/>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
             <c:v>Revenue (GBP)</c:v>
           </c:tx>
           <c:marker>
@@ -365,106 +337,6 @@
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <c:chart>
-    <c:plotArea>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:v>Series 1</c:v>
-          </c:tx>
-          <c:cat>
-            <c:strLit>
-              <c:ptCount val="1"/>
-              <c:pt idx="0">
-                <c:v>Item 1</c:v>
-              </c:pt>
-            </c:strLit>
-          </c:cat>
-          <c:val>
-            <c:numLit>
-              <c:formatCode>General</c:formatCode>
-              <c:ptCount val="1"/>
-              <c:pt idx="0">
-                <c:v>0</c:v>
-              </c:pt>
-            </c:numLit>
-          </c:val>
-        </c:ser>
-        <c:axId val="48650112"/>
-        <c:axId val="48672768"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="48650112"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="48672768"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="48672768"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="CCCCCC"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:crossAx val="48650112"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-  </c:chart>
-  <c:spPr>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-      <a:solidFill>
-        <a:srgbClr val="D9D9D9"/>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-    </a:ln>
-  </c:spPr>
-</c:chartSpace>
-</file>
-
-<file path=xl/drawings/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <c:chart>
     <c:title>
       <c:tx>
         <c:rich>
@@ -483,6 +355,30 @@
       <c:barChart>
         <c:barDir val="col"/>
         <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Revenue (GBP)</c:v>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Customer Segments'!$A$4:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="0"/>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Customer Segments'!$E$4:$E$10</c:f>
+              <c:numCache>
+                <c:formatCode>£#,##0</c:formatCode>
+                <c:ptCount val="0"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
         <c:axId val="48650112"/>
         <c:axId val="48672768"/>
       </c:barChart>
@@ -576,37 +472,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rab34525478344b15"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" x="0" y="0"/>
-        <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R62c37255d49b4c67"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc1f67de9bc704e30"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -627,7 +493,7 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart"/>
+        <xdr:cNvPr id="2" name="Chart"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -636,7 +502,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcf1d97e2a25f4089"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R858b2257a9974bc2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -890,16 +756,16 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="24" t="n">
-        <x:f>SUM('Monthly Trend'!C4:C16)</x:f>
-        <x:v>10666684.544</x:v>
+        <x:f>ROUND(SUM('Monthly Trend'!C4:C16),0)</x:f>
+        <x:v>10666685</x:v>
       </x:c>
       <x:c r="C5" s="27" t="n">
         <x:f>SUM('Monthly Trend'!D4:D16)</x:f>
         <x:v>19960</x:v>
       </x:c>
       <x:c r="E5" s="24" t="n">
-        <x:f>A5/C5</x:f>
-        <x:v>534.403033266533</x:v>
+        <x:f>ROUND(A5/C5,0)</x:f>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="G5" s="27" t="n">
         <x:f>SUM('Customer Segments'!B4:B10)</x:f>
@@ -975,7 +841,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2281f056cae044dc"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8fe6b7fc4ec4a03"/>
 </x:worksheet>
 </file>
 

</xml_diff>